<commit_message>
multi delete receipts implemented
</commit_message>
<xml_diff>
--- a/Receipts_data.xlsx
+++ b/Receipts_data.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\hasan\npo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4002237C-1C97-4DFD-91A0-E41638AEFE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93EDC83C-9FC0-49D4-986B-924D1C4EDE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{544B1080-0137-4549-8B03-49DF3A5BF1E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$299</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -9102,6 +9105,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I299" xr:uid="{BD13D3A8-7DE2-4CA1-9EA5-47A74B93BDF0}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>